<commit_message>
Module 1: remove the Named Ranges subsection (info overload); drop its reference from the weighted-average example
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/Sask_barley_varieties_2025.xlsx
+++ b/textbook_examples/Sask_barley_varieties_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B183F83-6EA1-2F46-B9F0-84E685C45A6C}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FC5573B-DEA5-5F4D-8A81-6003FDC9677D}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="2380" windowWidth="27640" windowHeight="18120" activeTab="2" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="51">
   <si>
     <t>Variety</t>
   </si>
@@ -179,6 +179,15 @@
   </si>
   <si>
     <t>We want to calculate total production of each variety and the revenue from each vareity, assuming a price of $5.50</t>
+  </si>
+  <si>
+    <t>Median</t>
+  </si>
+  <si>
+    <t>Median (formula)</t>
+  </si>
+  <si>
+    <t>Variability in yields by variety</t>
   </si>
 </sst>
 </file>
@@ -833,7 +842,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -877,6 +886,7 @@
     <xf numFmtId="0" fontId="21" fillId="35" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="35" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1667,7 +1677,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3FA5E1E-6B20-534B-92DF-F299182CFC14}">
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" customWidth="1"/>
@@ -2674,6 +2684,39 @@
       <c r="F42" s="26"/>
       <c r="G42" s="28"/>
     </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" s="29"/>
+      <c r="C44" s="30">
+        <f ca="1">MEDIAN(C8:C39)</f>
+        <v>84.1</v>
+      </c>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="31"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B45" s="32"/>
+      <c r="C45" s="32" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C44)</f>
+        <v>=MEDIAN(C8:C39)</v>
+      </c>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="33"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="35" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C33">
     <sortCondition ref="A2:A33"/>

</xml_diff>

<commit_message>
Module 1: move Charts to 1.7 as 'Visualizing the Shape of the Data'; keep histograms and box plots, defer bar/line/pie to Module 4
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/Sask_barley_varieties_2025.xlsx
+++ b/textbook_examples/Sask_barley_varieties_2025.xlsx
@@ -8,15 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FC5573B-DEA5-5F4D-8A81-6003FDC9677D}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{710CE71C-45A5-1C40-A9D5-8DB17BF488B3}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2380" windowWidth="27640" windowHeight="18120" activeTab="2" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
+    <workbookView xWindow="1620" yWindow="900" windowWidth="27640" windowHeight="18120" activeTab="2" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Raw_data" sheetId="2" r:id="rId2"/>
     <sheet name="Calculated_data" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Calculated_data!$J$12</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Calculated_data!$C$2:$C$33</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Calculated_data!$C$2:$C$33</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Calculated_data!$C$2:$C$33</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -35,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="57">
   <si>
     <t>Variety</t>
   </si>
@@ -187,7 +194,46 @@
     <t>Median (formula)</t>
   </si>
   <si>
-    <t>Variability in yields by variety</t>
+    <t>Coefficient of variation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A note on interpreting variability: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">correlation is not casuation!  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The fact that some barley varieties perform worse than others might be due to the varieties themselves.  But is could also be due to the type of farmers that grown them.  Maybe some varieties are a bit more drought tolerant than others.  So farmers who face drought are more likely to use these varieties.  This means that there isn't a fair comparison between varieties. </t>
+    </r>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Spread of varietal yields</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>Variance</t>
+  </si>
+  <si>
+    <t>Standard deviation</t>
   </si>
 </sst>
 </file>
@@ -842,7 +888,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -886,7 +932,46 @@
     <xf numFmtId="0" fontId="21" fillId="35" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="35" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -943,6 +1028,689 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.1</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0"/>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-5D3A-1744-918C-62045F5D4A2E}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:endParaRPr>
+          </a:p>
+        </cx:txPr>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Chart 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49497F0E-D2BD-1332-556B-213E2BC0AC76}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4432300" y="2603500"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1677,10 +2445,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3FA5E1E-6B20-534B-92DF-F299182CFC14}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.1640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -2714,16 +3482,143 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="B47" s="36"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="E47" s="37"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="38"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="40"/>
+      <c r="C48" s="41">
+        <f>MAX(C2:C33)-MIN(C2:C33)</f>
+        <v>85.5</v>
+      </c>
+      <c r="D48" s="40" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C48)</f>
+        <v>=MAX(C2:C33)-MIN(C2:C33)</v>
+      </c>
+      <c r="E48" s="42"/>
+      <c r="F48" s="40"/>
+      <c r="G48" s="43"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="B49" s="40"/>
+      <c r="C49" s="40">
+        <f>_xlfn.VAR.S(C2:C33)</f>
+        <v>350.52221774193362</v>
+      </c>
+      <c r="D49" s="40" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C49)</f>
+        <v>=VAR.S(C2:C33)</v>
+      </c>
+      <c r="E49" s="42"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="43"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50" s="40"/>
+      <c r="C50" s="40">
+        <f>_xlfn.STDEV.S(C2:C33)</f>
+        <v>18.722238587891503</v>
+      </c>
+      <c r="D50" s="40" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C50)</f>
+        <v>=STDEV.S(C2:C33)</v>
+      </c>
+      <c r="E50" s="42"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="43"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" s="44" t="s">
         <v>50</v>
       </c>
+      <c r="B51" s="45"/>
+      <c r="C51" s="45">
+        <f>C50/C38</f>
+        <v>0.23455940600286901</v>
+      </c>
+      <c r="D51" s="45" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C51)</f>
+        <v>=C50/C38</v>
+      </c>
+      <c r="E51" s="46"/>
+      <c r="F51" s="45"/>
+      <c r="G51" s="47"/>
+    </row>
+    <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="B53" s="49"/>
+      <c r="C53" s="49"/>
+      <c r="D53" s="49"/>
+      <c r="E53" s="49"/>
+      <c r="F53" s="49"/>
+      <c r="G53" s="50"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" s="51"/>
+      <c r="B54" s="52"/>
+      <c r="C54" s="52"/>
+      <c r="D54" s="52"/>
+      <c r="E54" s="52"/>
+      <c r="F54" s="52"/>
+      <c r="G54" s="53"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" s="51"/>
+      <c r="B55" s="52"/>
+      <c r="C55" s="52"/>
+      <c r="D55" s="52"/>
+      <c r="E55" s="52"/>
+      <c r="F55" s="52"/>
+      <c r="G55" s="53"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" s="54"/>
+      <c r="B56" s="55"/>
+      <c r="C56" s="55"/>
+      <c r="D56" s="55"/>
+      <c r="E56" s="55"/>
+      <c r="F56" s="55"/>
+      <c r="G56" s="56"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C33">
     <sortCondition ref="A2:A33"/>
   </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="A53:G56"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError sqref="F2:F33" formula="1"/>
   </ignoredErrors>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4699588-C4C7-8A47-A191-4CCEDE844128}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Module 1: add dot-chart figures for spread (wide/tight/hail) and distribution shape (bimodal/unimodal); resolve figure placeholders
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/Sask_barley_varieties_2025.xlsx
+++ b/textbook_examples/Sask_barley_varieties_2025.xlsx
@@ -8,21 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{710CE71C-45A5-1C40-A9D5-8DB17BF488B3}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51A4EEE3-DE4D-2348-8733-3B89D4BE7247}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="900" windowWidth="27640" windowHeight="18120" activeTab="2" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
+    <workbookView xWindow="1620" yWindow="900" windowWidth="27640" windowHeight="18120" activeTab="4" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Raw_data" sheetId="2" r:id="rId2"/>
     <sheet name="Calculated_data" sheetId="1" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
+    <sheet name="Histogram" sheetId="4" r:id="rId4"/>
+    <sheet name="Box_whisker_plot" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Calculated_data!$J$12</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Calculated_data!$C$2:$C$33</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Calculated_data!$C$2:$C$33</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Calculated_data!$C$2:$C$33</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Calculated_data!$C$2:$C$33</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Box_whisker_plot!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Box_whisker_plot!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Box_whisker_plot!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Box_whisker_plot!$A$3:$A$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="56">
   <si>
     <t>Variety</t>
   </si>
@@ -180,12 +185,6 @@
   </si>
   <si>
     <t>Weighted average (formula)</t>
-  </si>
-  <si>
-    <t>This workbook contains raw data on acreage and average yields of Barley varieties in Saskatchewan in 2025</t>
-  </si>
-  <si>
-    <t>We want to calculate total production of each variety and the revenue from each vareity, assuming a price of $5.50</t>
   </si>
   <si>
     <t>Median</t>
@@ -235,6 +234,9 @@
   <si>
     <t>Standard deviation</t>
   </si>
+  <si>
+    <t>This workbook contains raw data on acreage and average yields of Barley varieties in Saskatchewan in 2025 and summary statistics of the data</t>
+  </si>
 </sst>
 </file>
 
@@ -243,7 +245,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -401,6 +403,13 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
@@ -888,7 +897,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -900,9 +909,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -972,6 +978,15 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="34" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1040,27 +1055,84 @@
     </cx:data>
   </cx:chartData>
   <cx:chart>
-    <cx:title pos="t" align="ctr" overlay="0"/>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Histogram of Average Saskatchewan Barley Variety Yields  in 2025</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1600"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:rPr>
+            <a:t>Histogram of Average Saskatchewan Barley Variety Yields  in 2025</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
-        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-5D3A-1744-918C-62045F5D4A2E}">
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-0544-1644-87B6-0D2A04D2962F}">
           <cx:dataId val="0"/>
           <cx:layoutPr>
-            <cx:binning intervalClosed="r"/>
+            <cx:binning intervalClosed="r" underflow="40" overflow="100">
+              <cx:binSize val="15"/>
+            </cx:binning>
           </cx:layoutPr>
         </cx:series>
       </cx:plotAreaRegion>
       <cx:axis id="0">
         <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Average yield of variety (bu/acre)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Average yield of variety (bu/acre)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:tickLabels/>
         <cx:txPr>
           <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:sysClr val="windowText" lastClr="000000">
                   <a:lumMod val="65000"/>
@@ -1074,6 +1146,184 @@
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count of barley varieties</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count of barley varieties</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.5</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Box and Whisker Plot of Saskatchewan Average Barley Variety Yields in 2026</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1600"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:rPr>
+            <a:t>Box and Whisker Plot of Saskatchewan Average Barley Variety Yields in 2026</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000000-D8B4-8D48-8E58-3375C50C4539}">
+          <cx:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </cx:spPr>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0" hidden="1">
+        <cx:catScaling gapWidth="1"/>
+        <cx:title>
+          <cx:tx>
+            <cx:rich>
+              <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr algn="ctr" rtl="0">
+                  <a:defRPr sz="1200"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                  </a:rPr>
+                  <a:t>The upper and lower bounds of the box represent the first and third quartile of the data.  </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                    <a:effectLst/>
+                    <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                    <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>The line and X within the box represent the mean and median of the data respectively.  </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                    <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                  </a:rPr>
+                  <a:t>The whiskers of the plot represent the most exterem values within 1.5 time the interquartile range from the mean.  The dots represent outliers.</a:t>
+                </a:r>
+              </a:p>
+            </cx:rich>
+          </cx:tx>
+        </cx:title>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Yields in Busehls per Acre</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Yields in Busehls per Acre</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
@@ -1122,6 +1372,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -1630,29 +1920,544 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="4" name="Chart 3">
+            <xdr:cNvPr id="3" name="Chart 2">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49497F0E-D2BD-1332-556B-213E2BC0AC76}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44BC997D-FE97-B0EC-404D-89C14BFF3E1E}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1679,8 +2484,91 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="4432300" y="2603500"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="2298700" y="596900"/>
+              <a:ext cx="7505700" cy="4597400"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>812800</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71E449F1-58F0-5BC2-FD72-32789DAB3275}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4432300" y="927100"/>
+              <a:ext cx="4635500" cy="5003800"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2030,41 +2918,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{952F3771-09AC-AA47-B5A6-E67DCD85978C}">
-  <dimension ref="A5:J7"/>
+  <dimension ref="A5:J8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="5" spans="1:10" ht="47" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-    </row>
-    <row r="7" spans="1:10" ht="47" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-    </row>
+      <c r="A5" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+    </row>
+    <row r="7" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="58"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58"/>
+      <c r="I7" s="58"/>
+      <c r="J7" s="58"/>
+    </row>
+    <row r="8" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A7:J7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2076,365 +2962,365 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="60" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="60">
         <v>392684</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="60">
         <v>86.6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="60">
         <v>197626</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="60">
         <v>76.099999999999994</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="60">
         <v>143023</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="60">
         <v>90.1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="60">
         <v>125867</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="60">
         <v>84.8</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="60">
         <v>74958</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="60">
         <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="60">
         <v>66119</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="60">
         <v>93.7</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="60">
         <v>55767</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="60">
         <v>48.3</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="60">
         <v>38961</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="60">
         <v>87.4</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="60">
         <v>22568</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="60">
         <v>75.7</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="60">
         <v>21676</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="60">
         <v>77.099999999999994</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="60">
         <v>21311</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="60">
         <v>95.9</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="A13" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="60">
         <v>18710</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="60">
         <v>96.7</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="60">
         <v>17566</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="60">
         <v>66.900000000000006</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="60">
         <v>10249</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="60">
         <v>40.5</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="A16" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="60">
         <v>8884</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="60">
         <v>55.9</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="A17" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="60">
         <v>7282</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="60">
         <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="A18" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="60">
         <v>6754</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="60">
         <v>97.1</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="A19" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="60">
         <v>5792</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="60">
         <v>72.5</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="A20" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="60">
         <v>5636</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="60">
         <v>102.6</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="A21" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="60">
         <v>5274</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="60">
         <v>84.1</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="A22" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="60">
         <v>5090</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="60">
         <v>56.9</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="A23" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="60">
         <v>4750</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="60">
         <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="A24" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="60">
         <v>3015</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="60">
         <v>39.200000000000003</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="A25" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="60">
         <v>2607</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="60">
         <v>124.7</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="A26" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="60">
         <v>2190</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="60">
         <v>89.1</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="A27" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="60">
         <v>1998</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="60">
         <v>97.5</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="A28" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="60">
         <v>1430</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="60">
         <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="A29" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="60">
         <v>1287</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="60">
         <v>56.5</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="A30" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="60">
         <v>901</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="60">
         <v>79.2</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="A31" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="60">
         <v>825</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="60">
         <v>79.2</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="A32" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="60">
         <v>700</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="60">
         <v>80.099999999999994</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="A33" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="60">
         <v>460</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="60">
         <v>90.8</v>
       </c>
     </row>
@@ -2458,36 +3344,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="19" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="12">
         <v>22568</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="13">
         <v>75.7</v>
       </c>
       <c r="D2" s="2">
@@ -2514,13 +3400,13 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="12">
         <v>700</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="13">
         <v>80.099999999999994</v>
       </c>
       <c r="D3" s="2">
@@ -2541,13 +3427,13 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="12">
         <v>18710</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="13">
         <v>96.7</v>
       </c>
       <c r="D4" s="2">
@@ -2568,13 +3454,13 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="12">
         <v>197626</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="13">
         <v>76.099999999999994</v>
       </c>
       <c r="D5" s="2">
@@ -2595,13 +3481,13 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="12">
         <v>2607</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="13">
         <v>124.7</v>
       </c>
       <c r="D6" s="2">
@@ -2622,13 +3508,13 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="12">
         <v>5792</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="13">
         <v>72.5</v>
       </c>
       <c r="D7" s="2">
@@ -2649,13 +3535,13 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="12">
         <v>1998</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="13">
         <v>97.5</v>
       </c>
       <c r="D8" s="2">
@@ -2676,13 +3562,13 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="12">
         <v>8884</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="13">
         <v>55.9</v>
       </c>
       <c r="D9" s="2">
@@ -2703,13 +3589,13 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="12">
         <v>66119</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="13">
         <v>93.7</v>
       </c>
       <c r="D10" s="2">
@@ -2730,13 +3616,13 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="12">
         <v>21676</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="13">
         <v>77.099999999999994</v>
       </c>
       <c r="D11" s="2">
@@ -2757,13 +3643,13 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="12">
         <v>5274</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="13">
         <v>84.1</v>
       </c>
       <c r="D12" s="2">
@@ -2784,13 +3670,13 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="12">
         <v>143023</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="13">
         <v>90.1</v>
       </c>
       <c r="D13" s="2">
@@ -2811,13 +3697,13 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14" s="12">
         <v>125867</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="13">
         <v>84.8</v>
       </c>
       <c r="D14" s="2">
@@ -2838,13 +3724,13 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="12">
         <v>901</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="13">
         <v>79.2</v>
       </c>
       <c r="D15" s="2">
@@ -2865,13 +3751,13 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="13">
+      <c r="B16" s="12">
         <v>10249</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="13">
         <v>40.5</v>
       </c>
       <c r="D16" s="2">
@@ -2892,13 +3778,13 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="12">
         <v>38961</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="13">
         <v>87.4</v>
       </c>
       <c r="D17" s="2">
@@ -2919,13 +3805,13 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="12">
         <v>6754</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="13">
         <v>97.1</v>
       </c>
       <c r="D18" s="2">
@@ -2946,13 +3832,13 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="12">
         <v>74958</v>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="13">
         <v>88</v>
       </c>
       <c r="D19" s="2">
@@ -2973,13 +3859,13 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="12">
         <v>7282</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="13">
         <v>96</v>
       </c>
       <c r="D20" s="2">
@@ -3000,13 +3886,13 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="12">
         <v>4750</v>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="13">
         <v>73</v>
       </c>
       <c r="D21" s="2">
@@ -3027,13 +3913,13 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="12">
         <v>21311</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="13">
         <v>95.9</v>
       </c>
       <c r="D22" s="2">
@@ -3054,13 +3940,13 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="12">
         <v>55767</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="13">
         <v>48.3</v>
       </c>
       <c r="D23" s="2">
@@ -3081,13 +3967,13 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="12">
         <v>825</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="13">
         <v>79.2</v>
       </c>
       <c r="D24" s="2">
@@ -3108,13 +3994,13 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="13">
+      <c r="B25" s="12">
         <v>5090</v>
       </c>
-      <c r="C25" s="14">
+      <c r="C25" s="13">
         <v>56.9</v>
       </c>
       <c r="D25" s="2">
@@ -3135,13 +4021,13 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="12">
         <v>2190</v>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="13">
         <v>89.1</v>
       </c>
       <c r="D26" s="2">
@@ -3162,13 +4048,13 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="12">
         <v>5636</v>
       </c>
-      <c r="C27" s="14">
+      <c r="C27" s="13">
         <v>102.6</v>
       </c>
       <c r="D27" s="2">
@@ -3189,13 +4075,13 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="12">
         <v>460</v>
       </c>
-      <c r="C28" s="14">
+      <c r="C28" s="13">
         <v>90.8</v>
       </c>
       <c r="D28" s="2">
@@ -3216,13 +4102,13 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B29" s="13">
+      <c r="B29" s="12">
         <v>17566</v>
       </c>
-      <c r="C29" s="14">
+      <c r="C29" s="13">
         <v>66.900000000000006</v>
       </c>
       <c r="D29" s="2">
@@ -3243,13 +4129,13 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="12">
         <v>1430</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="13">
         <v>72</v>
       </c>
       <c r="D30" s="2">
@@ -3270,13 +4156,13 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="12">
         <v>392684</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="13">
         <v>86.6</v>
       </c>
       <c r="D31" s="2">
@@ -3297,13 +4183,13 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="13">
+      <c r="B32" s="12">
         <v>3015</v>
       </c>
-      <c r="C32" s="14">
+      <c r="C32" s="13">
         <v>39.200000000000003</v>
       </c>
       <c r="D32" s="2">
@@ -3324,13 +4210,13 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="16">
+      <c r="B33" s="15">
         <v>1287</v>
       </c>
-      <c r="C33" s="17">
+      <c r="C33" s="16">
         <v>56.5</v>
       </c>
       <c r="D33" s="5">
@@ -3351,253 +4237,253 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="B35" s="22">
+      <c r="B35" s="21">
         <f>SUM(B1:B33)</f>
         <v>1271960</v>
       </c>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22">
+      <c r="C35" s="21"/>
+      <c r="D35" s="21">
         <f>SUM(D1:D33)</f>
         <v>105491924.29999998</v>
       </c>
-      <c r="E35" s="23"/>
-      <c r="F35" s="22">
+      <c r="E35" s="22"/>
+      <c r="F35" s="21">
         <f>SUM(F1:F33)</f>
         <v>580205583.64999998</v>
       </c>
-      <c r="G35" s="24"/>
+      <c r="G35" s="23"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="25" t="s">
+      <c r="A36" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="B36" s="26" t="str">
+      <c r="B36" s="25" t="str">
         <f ca="1">_xlfn.FORMULATEXT(B35)</f>
         <v>=SUM(B1:B33)</v>
       </c>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26" t="str">
+      <c r="C36" s="25"/>
+      <c r="D36" s="25" t="str">
         <f ca="1">_xlfn.FORMULATEXT(D35)</f>
         <v>=SUM(D1:D33)</v>
       </c>
-      <c r="E36" s="27"/>
-      <c r="F36" s="26" t="str">
+      <c r="E36" s="26"/>
+      <c r="F36" s="25" t="str">
         <f ca="1">_xlfn.FORMULATEXT(F35)</f>
         <v>=SUM(F1:F33)</v>
       </c>
-      <c r="G36" s="28"/>
+      <c r="G36" s="27"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="8"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="21" t="s">
+      <c r="A38" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="29"/>
-      <c r="C38" s="30">
+      <c r="B38" s="28"/>
+      <c r="C38" s="29">
         <f>AVERAGE(C2:C33)</f>
         <v>79.818750000000009</v>
       </c>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="31"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="30"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32" t="str">
+      <c r="B39" s="31"/>
+      <c r="C39" s="31" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C38)</f>
         <v>=AVERAGE(C2:C33)</v>
       </c>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="33"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="32"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="8"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="21" t="s">
+      <c r="A41" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="22"/>
-      <c r="C41" s="34">
+      <c r="B41" s="21"/>
+      <c r="C41" s="33">
         <f>SUMPRODUCT(C2:C33,B2:B33)/SUM(B2:B33)</f>
         <v>82.936510817950236</v>
       </c>
-      <c r="D41" s="22"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="24"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="23"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="26"/>
-      <c r="C42" s="26" t="str">
+      <c r="B42" s="25"/>
+      <c r="C42" s="25" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C41)</f>
         <v>=SUMPRODUCT(C2:C33,B2:B33)/SUM(B2:B33)</v>
       </c>
-      <c r="D42" s="26"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="28"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="26"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="27"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B44" s="29"/>
-      <c r="C44" s="30">
+      <c r="A44" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="28"/>
+      <c r="C44" s="29">
         <f ca="1">MEDIAN(C8:C39)</f>
         <v>84.1</v>
       </c>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="31"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
+      <c r="G44" s="30"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32" t="str">
+      <c r="A45" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="31"/>
+      <c r="C45" s="31" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C44)</f>
         <v>=MEDIAN(C8:C39)</v>
       </c>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="33"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
+      <c r="F45" s="31"/>
+      <c r="G45" s="32"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="B47" s="36"/>
-      <c r="C47" s="36"/>
-      <c r="D47" s="36" t="s">
+      <c r="A47" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="E47" s="36"/>
+      <c r="F47" s="35"/>
+      <c r="G47" s="37"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="E47" s="37"/>
-      <c r="F47" s="36"/>
-      <c r="G47" s="38"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="39" t="s">
-        <v>54</v>
-      </c>
-      <c r="B48" s="40"/>
-      <c r="C48" s="41">
+      <c r="B48" s="39"/>
+      <c r="C48" s="40">
         <f>MAX(C2:C33)-MIN(C2:C33)</f>
         <v>85.5</v>
       </c>
-      <c r="D48" s="40" t="str">
+      <c r="D48" s="39" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C48)</f>
         <v>=MAX(C2:C33)-MIN(C2:C33)</v>
       </c>
-      <c r="E48" s="42"/>
-      <c r="F48" s="40"/>
-      <c r="G48" s="43"/>
+      <c r="E48" s="41"/>
+      <c r="F48" s="39"/>
+      <c r="G48" s="42"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="39" t="s">
-        <v>55</v>
-      </c>
-      <c r="B49" s="40"/>
-      <c r="C49" s="40">
+      <c r="A49" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="B49" s="39"/>
+      <c r="C49" s="39">
         <f>_xlfn.VAR.S(C2:C33)</f>
         <v>350.52221774193362</v>
       </c>
-      <c r="D49" s="40" t="str">
+      <c r="D49" s="39" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C49)</f>
         <v>=VAR.S(C2:C33)</v>
       </c>
-      <c r="E49" s="42"/>
-      <c r="F49" s="40"/>
-      <c r="G49" s="43"/>
+      <c r="E49" s="41"/>
+      <c r="F49" s="39"/>
+      <c r="G49" s="42"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="40"/>
-      <c r="C50" s="40">
+      <c r="A50" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50" s="39"/>
+      <c r="C50" s="39">
         <f>_xlfn.STDEV.S(C2:C33)</f>
         <v>18.722238587891503</v>
       </c>
-      <c r="D50" s="40" t="str">
+      <c r="D50" s="39" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C50)</f>
         <v>=STDEV.S(C2:C33)</v>
       </c>
-      <c r="E50" s="42"/>
-      <c r="F50" s="40"/>
-      <c r="G50" s="43"/>
+      <c r="E50" s="41"/>
+      <c r="F50" s="39"/>
+      <c r="G50" s="42"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A51" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="B51" s="45"/>
-      <c r="C51" s="45">
+      <c r="A51" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" s="44"/>
+      <c r="C51" s="44">
         <f>C50/C38</f>
         <v>0.23455940600286901</v>
       </c>
-      <c r="D51" s="45" t="str">
+      <c r="D51" s="44" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C51)</f>
         <v>=C50/C38</v>
       </c>
-      <c r="E51" s="46"/>
-      <c r="F51" s="45"/>
-      <c r="G51" s="47"/>
+      <c r="E51" s="45"/>
+      <c r="F51" s="44"/>
+      <c r="G51" s="46"/>
     </row>
     <row r="53" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="B53" s="49"/>
-      <c r="C53" s="49"/>
-      <c r="D53" s="49"/>
-      <c r="E53" s="49"/>
-      <c r="F53" s="49"/>
-      <c r="G53" s="50"/>
+      <c r="A53" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" s="48"/>
+      <c r="C53" s="48"/>
+      <c r="D53" s="48"/>
+      <c r="E53" s="48"/>
+      <c r="F53" s="48"/>
+      <c r="G53" s="49"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A54" s="51"/>
-      <c r="B54" s="52"/>
-      <c r="C54" s="52"/>
-      <c r="D54" s="52"/>
-      <c r="E54" s="52"/>
-      <c r="F54" s="52"/>
-      <c r="G54" s="53"/>
+      <c r="A54" s="50"/>
+      <c r="B54" s="51"/>
+      <c r="C54" s="51"/>
+      <c r="D54" s="51"/>
+      <c r="E54" s="51"/>
+      <c r="F54" s="51"/>
+      <c r="G54" s="52"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55" s="51"/>
-      <c r="B55" s="52"/>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="53"/>
+      <c r="A55" s="50"/>
+      <c r="B55" s="51"/>
+      <c r="C55" s="51"/>
+      <c r="D55" s="51"/>
+      <c r="E55" s="51"/>
+      <c r="F55" s="51"/>
+      <c r="G55" s="52"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" s="54"/>
-      <c r="B56" s="55"/>
-      <c r="C56" s="55"/>
-      <c r="D56" s="55"/>
-      <c r="E56" s="55"/>
-      <c r="F56" s="55"/>
-      <c r="G56" s="56"/>
+      <c r="A56" s="53"/>
+      <c r="B56" s="54"/>
+      <c r="C56" s="54"/>
+      <c r="D56" s="54"/>
+      <c r="E56" s="54"/>
+      <c r="F56" s="54"/>
+      <c r="G56" s="55"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C33">
@@ -3610,15 +4496,357 @@
   <ignoredErrors>
     <ignoredError sqref="F2:F33" formula="1"/>
   </ignoredErrors>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4699588-C4C7-8A47-A191-4CCEDE844128}">
-  <dimension ref="A1"/>
+  <dimension ref="A2:A34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="12">
+        <v>75.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="12">
+        <v>80.099999999999994</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="12">
+        <v>96.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12">
+        <v>76.099999999999994</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="12">
+        <v>124.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="12">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="12">
+        <v>97.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="12">
+        <v>55.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="12">
+        <v>93.7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="12">
+        <v>77.099999999999994</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12">
+        <v>84.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="12">
+        <v>90.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="12">
+        <v>84.8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="12">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="12">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="12">
+        <v>87.4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="12">
+        <v>97.1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="12">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="12">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="12">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="12">
+        <v>95.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="12">
+        <v>48.3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="12">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="12">
+        <v>56.9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="12">
+        <v>89.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="12">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="12">
+        <v>90.8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="12">
+        <v>66.900000000000006</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="12">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="12">
+        <v>86.6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="12">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="15">
+        <v>56.5</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD2D9963-5988-1C43-9E23-4BD45B1135D5}">
+  <dimension ref="A2:A34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="56">
+        <v>75.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="56">
+        <v>80.099999999999994</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="56">
+        <v>96.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="56">
+        <v>76.099999999999994</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="56">
+        <v>124.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="56">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="56">
+        <v>97.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="56">
+        <v>55.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="56">
+        <v>93.7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="56">
+        <v>77.099999999999994</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="56">
+        <v>84.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="56">
+        <v>90.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="56">
+        <v>84.8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="56">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="56">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="56">
+        <v>87.4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="56">
+        <v>97.1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="56">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="56">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="56">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="56">
+        <v>95.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="56">
+        <v>48.3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="56">
+        <v>79.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="56">
+        <v>56.9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="56">
+        <v>89.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="56">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="56">
+        <v>90.8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="56">
+        <v>66.900000000000006</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="56">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="56">
+        <v>86.6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="56">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="57">
+        <v>56.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reorder the test bank to follow the teaching sequence
Section 1 is now Building a Worksheet (the Module 1a mechanics), 2 is
Descriptive Statistics, 3 is Conditional Functions and Lookups, 4 is
PivotTables. Questions renumber continuously 1-100.

The twenty leftover chart questions are parked in
practice/_parked_chart_questions.md rather than deleted -- several are
histogram questions that belong in Section 2 once reworked.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/Sask_barley_varieties_2025.xlsx
+++ b/textbook_examples/Sask_barley_varieties_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="340" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33F12D39-3FF1-6E49-89F4-058A6CDE3FEE}"/>
+  <xr:revisionPtr revIDLastSave="351" documentId="8_{E03AF2A9-D327-A541-ADB2-E7D79CDD9711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F4D7398-F796-CE4E-A558-C1021502C8CD}"/>
   <bookViews>
     <workbookView xWindow="1620" yWindow="900" windowWidth="27640" windowHeight="18120" activeTab="5" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
   </bookViews>
@@ -22,6 +22,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Histogram!$A$3:$A$34</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Histogram!$A$3:$A$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1138,7 +1142,393 @@
 </cx:chartSpace>
 </file>
 
+<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.1</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:rich>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1600"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+              </a:rPr>
+              <a:t>Histogram of Average Saskatchewan Barley Variety Yields  in 2025 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+              </a:rPr>
+              <a:t>(too many bins)</a:t>
+            </a:r>
+          </a:p>
+        </cx:rich>
+      </cx:tx>
+      <cx:extLst>
+        <cx:ext uri="ext:featex">
+          <cx:featureExtension feature="mp" drop="onModelChange">
+            <cx:offset top="-0.013888888992369175" left="0.4861111044883728"/>
+          </cx:featureExtension>
+        </cx:ext>
+      </cx:extLst>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-0544-1644-87B6-0D2A04D2962F}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r" underflow="40" overflow="100">
+              <cx:binSize val="5"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Average yield of variety (bu/acre)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Average yield of variety (bu/acre)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:endParaRPr>
+          </a:p>
+        </cx:txPr>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count of barley varieties</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count of barley varieties</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx3.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.3</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:rich>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1600"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+              </a:rPr>
+              <a:t>Histogram of Average Saskatchewan Barley Variety Yields  in 2025 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+              </a:rPr>
+              <a:t>(too few bins)</a:t>
+            </a:r>
+          </a:p>
+        </cx:rich>
+      </cx:tx>
+      <cx:extLst>
+        <cx:ext uri="ext:featex">
+          <cx:featureExtension feature="mp" drop="onModelChange">
+            <cx:offset top="-0.013888888992369175" left="0.4861111044883728"/>
+          </cx:featureExtension>
+        </cx:ext>
+      </cx:extLst>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-0544-1644-87B6-0D2A04D2962F}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r" underflow="40" overflow="100">
+              <cx:binSize val="30"/>
+            </cx:binning>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Average yield of variety (bu/acre)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Average yield of variety (bu/acre)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:endParaRPr>
+          </a:p>
+        </cx:txPr>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Count of barley varieties</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1200"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Count of barley varieties</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1686,20 +2076,1036 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>723900</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>279400</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
@@ -1735,8 +3141,164 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="2298700" y="596900"/>
-              <a:ext cx="7505700" cy="4597400"/>
+              <a:off x="901700" y="88900"/>
+              <a:ext cx="5156200" cy="2794000"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>292100</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFB31C8C-0379-084B-A55F-BDB20F5AA586}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="914400" y="2959100"/>
+              <a:ext cx="5156200" cy="2794000"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>101600</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Chart 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EDDA579-0314-8448-AF02-DE074F6A209F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="927100" y="5803900"/>
+              <a:ext cx="5156200" cy="2794000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>

</xml_diff>

<commit_message>
Add module 4 bar and line chart workbooks (download targets for module04b embeds)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/Sask_barley_varieties_2025.xlsx
+++ b/textbook_examples/Sask_barley_varieties_2025.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -24,8 +24,6 @@
     <definedName name="_xlchart.v1.0" hidden="1">Histogram!$A$3:$A$34</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">Histogram!$A$3:$A$34</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">Histogram!$A$3:$A$34</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Histogram!$A$3:$A$34</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Histogram!$A$3:$A$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -902,7 +900,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="34" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -914,37 +912,35 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" xfId="42" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" xfId="42" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1300,7 +1296,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -3655,18 +3651,18 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:10" ht="47" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
     </row>
     <row r="7" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
@@ -3681,47 +3677,47 @@
       <c r="J7" s="5"/>
     </row>
     <row r="8" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="23"/>
     </row>
     <row r="9" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="20" t="s">
         <v>56</v>
       </c>
       <c r="B9" s="4"/>
     </row>
     <row r="10" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A10" s="27"/>
+      <c r="A10" s="21"/>
       <c r="B10" s="4"/>
     </row>
     <row r="11" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="21" t="s">
         <v>57</v>
       </c>
       <c r="B11" s="4"/>
     </row>
     <row r="12" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="4"/>
     </row>
     <row r="13" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="20" t="s">
         <v>59</v>
       </c>
       <c r="B13" s="4"/>
     </row>
     <row r="14" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="20" t="s">
         <v>60</v>
       </c>
       <c r="B14" s="4"/>
     </row>
     <row r="15" spans="1:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="20" t="s">
         <v>61</v>
       </c>
       <c r="B15" s="4"/>
@@ -4121,7 +4117,6 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="18"/>
     <col min="6" max="6" width="14.1640625" customWidth="1"/>
     <col min="7" max="7" width="10.6640625" customWidth="1"/>
     <col min="8" max="8" width="44.5" customWidth="1"/>
@@ -4137,7 +4132,7 @@
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4151,14 +4146,14 @@
       <c r="C2" s="6">
         <v>86.6</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="16">
         <f>B2*C2</f>
         <v>34006434.399999999</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="9"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -4170,14 +4165,14 @@
       <c r="C3" s="6">
         <v>76.099999999999994</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="16">
         <f t="shared" ref="D3:D33" si="0">B3*C3</f>
         <v>15039338.6</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="10">
         <f>AVERAGE(C2:C33)</f>
         <v>79.81874999999998</v>
       </c>
@@ -4196,14 +4191,14 @@
       <c r="C4" s="6">
         <v>90.1</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="16">
         <f t="shared" si="0"/>
         <v>12886372.299999999</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="12">
         <f>D34/B34</f>
         <v>82.93651081795025</v>
       </c>
@@ -4222,12 +4217,12 @@
       <c r="C5" s="6">
         <v>84.8</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="16">
         <f t="shared" si="0"/>
         <v>10673521.6</v>
       </c>
-      <c r="F5" s="14"/>
-      <c r="G5" s="15">
+      <c r="F5" s="11"/>
+      <c r="G5" s="12">
         <f>SUMPRODUCT(B2:B33,C2:C33)/SUM(B2:B33)</f>
         <v>82.93651081795025</v>
       </c>
@@ -4246,14 +4241,14 @@
       <c r="C6" s="6">
         <v>88</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="16">
         <f t="shared" si="0"/>
         <v>6596304</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="12">
         <f>MEDIAN(C2:C33)</f>
         <v>82.1</v>
       </c>
@@ -4272,14 +4267,14 @@
       <c r="C7" s="6">
         <v>93.7</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="16">
         <f t="shared" si="0"/>
         <v>6195350.2999999998</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="14">
         <f>MODE(C2:C33)</f>
         <v>79.2</v>
       </c>
@@ -4298,7 +4293,7 @@
       <c r="C8" s="6">
         <v>48.3</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="16">
         <f t="shared" si="0"/>
         <v>2693546.0999999996</v>
       </c>
@@ -4313,7 +4308,7 @@
       <c r="C9" s="6">
         <v>87.4</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="16">
         <f t="shared" si="0"/>
         <v>3405191.4000000004</v>
       </c>
@@ -4328,7 +4323,7 @@
       <c r="C10" s="6">
         <v>75.7</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="16">
         <f t="shared" si="0"/>
         <v>1708397.6</v>
       </c>
@@ -4343,7 +4338,7 @@
       <c r="C11" s="6">
         <v>77.099999999999994</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="16">
         <f t="shared" si="0"/>
         <v>1671219.5999999999</v>
       </c>
@@ -4358,7 +4353,7 @@
       <c r="C12" s="6">
         <v>95.9</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="16">
         <f t="shared" si="0"/>
         <v>2043724.9000000001</v>
       </c>
@@ -4373,7 +4368,7 @@
       <c r="C13" s="6">
         <v>96.7</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="16">
         <f t="shared" si="0"/>
         <v>1809257</v>
       </c>
@@ -4388,7 +4383,7 @@
       <c r="C14" s="6">
         <v>66.900000000000006</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="16">
         <f t="shared" si="0"/>
         <v>1175165.4000000001</v>
       </c>
@@ -4403,7 +4398,7 @@
       <c r="C15" s="6">
         <v>40.5</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="16">
         <f t="shared" si="0"/>
         <v>415084.5</v>
       </c>
@@ -4418,7 +4413,7 @@
       <c r="C16" s="6">
         <v>55.9</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="16">
         <f t="shared" si="0"/>
         <v>496615.6</v>
       </c>
@@ -4433,7 +4428,7 @@
       <c r="C17" s="6">
         <v>96</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="16">
         <f t="shared" si="0"/>
         <v>699072</v>
       </c>
@@ -4448,7 +4443,7 @@
       <c r="C18" s="6">
         <v>97.1</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="16">
         <f t="shared" si="0"/>
         <v>655813.39999999991</v>
       </c>
@@ -4463,7 +4458,7 @@
       <c r="C19" s="6">
         <v>72.5</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="16">
         <f t="shared" si="0"/>
         <v>419920</v>
       </c>
@@ -4478,7 +4473,7 @@
       <c r="C20" s="6">
         <v>102.6</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="16">
         <f t="shared" si="0"/>
         <v>578253.6</v>
       </c>
@@ -4493,7 +4488,7 @@
       <c r="C21" s="6">
         <v>84.1</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="16">
         <f t="shared" si="0"/>
         <v>443543.39999999997</v>
       </c>
@@ -4508,7 +4503,7 @@
       <c r="C22" s="6">
         <v>56.9</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="16">
         <f t="shared" si="0"/>
         <v>289621</v>
       </c>
@@ -4523,7 +4518,7 @@
       <c r="C23" s="6">
         <v>73</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="16">
         <f t="shared" si="0"/>
         <v>346750</v>
       </c>
@@ -4538,7 +4533,7 @@
       <c r="C24" s="6">
         <v>39.200000000000003</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="16">
         <f t="shared" si="0"/>
         <v>118188.00000000001</v>
       </c>
@@ -4553,7 +4548,7 @@
       <c r="C25" s="6">
         <v>124.7</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="16">
         <f t="shared" si="0"/>
         <v>325092.90000000002</v>
       </c>
@@ -4568,7 +4563,7 @@
       <c r="C26" s="6">
         <v>89.1</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="16">
         <f t="shared" si="0"/>
         <v>195129</v>
       </c>
@@ -4583,7 +4578,7 @@
       <c r="C27" s="6">
         <v>97.5</v>
       </c>
-      <c r="D27" s="20">
+      <c r="D27" s="16">
         <f t="shared" si="0"/>
         <v>194805</v>
       </c>
@@ -4598,7 +4593,7 @@
       <c r="C28" s="6">
         <v>72</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="16">
         <f t="shared" si="0"/>
         <v>102960</v>
       </c>
@@ -4613,7 +4608,7 @@
       <c r="C29" s="6">
         <v>56.5</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="16">
         <f t="shared" si="0"/>
         <v>72715.5</v>
       </c>
@@ -4628,7 +4623,7 @@
       <c r="C30" s="6">
         <v>79.2</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="16">
         <f t="shared" si="0"/>
         <v>71359.199999999997</v>
       </c>
@@ -4643,7 +4638,7 @@
       <c r="C31" s="6">
         <v>79.2</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="16">
         <f t="shared" si="0"/>
         <v>65340</v>
       </c>
@@ -4658,7 +4653,7 @@
       <c r="C32" s="6">
         <v>80.099999999999994</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="16">
         <f t="shared" si="0"/>
         <v>56069.999999999993</v>
       </c>
@@ -4673,21 +4668,21 @@
       <c r="C33" s="6">
         <v>90.8</v>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="16">
         <f t="shared" si="0"/>
         <v>41768</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="19">
+      <c r="B34" s="15">
         <f>SUM(B2:B33)</f>
         <v>1271960</v>
       </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="19">
+      <c r="C34" s="7"/>
+      <c r="D34" s="15">
         <f>SUM(D2:D33)</f>
         <v>105491924.3</v>
       </c>
@@ -4706,7 +4701,6 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="18"/>
     <col min="6" max="6" width="14.1640625" customWidth="1"/>
     <col min="7" max="7" width="10.6640625" customWidth="1"/>
     <col min="8" max="8" width="29.33203125" customWidth="1"/>
@@ -4722,7 +4716,7 @@
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4736,14 +4730,14 @@
       <c r="C2" s="6">
         <v>86.6</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="16">
         <f>B2*C2</f>
         <v>34006434.399999999</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="9"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -4755,14 +4749,14 @@
       <c r="C3" s="6">
         <v>76.099999999999994</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="16">
         <f t="shared" ref="D3:D33" si="0">B3*C3</f>
         <v>15039338.6</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="10">
         <f>_xlfn.QUARTILE.INC(C2:C33,1)</f>
         <v>72.375</v>
       </c>
@@ -4781,14 +4775,14 @@
       <c r="C4" s="6">
         <v>90.1</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="16">
         <f t="shared" si="0"/>
         <v>12886372.299999999</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="12">
         <f>_xlfn.QUARTILE.INC(C2:C33,3)</f>
         <v>91.525000000000006</v>
       </c>
@@ -4807,14 +4801,14 @@
       <c r="C5" s="6">
         <v>84.8</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="16">
         <f t="shared" si="0"/>
         <v>10673521.6</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="12">
         <f>_xlfn.PERCENTILE.INC(C2:C33, 0.1)</f>
         <v>55.96</v>
       </c>
@@ -4833,14 +4827,14 @@
       <c r="C6" s="6">
         <v>88</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="16">
         <f t="shared" si="0"/>
         <v>6596304</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="14">
         <f>_xlfn.PERCENTILE.INC(C2:C33,0.9)</f>
         <v>97.06</v>
       </c>
@@ -4859,12 +4853,11 @@
       <c r="C7" s="6">
         <v>93.7</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="16">
         <f t="shared" si="0"/>
         <v>6195350.2999999998</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="11"/>
+      <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
@@ -4876,15 +4869,15 @@
       <c r="C8" s="6">
         <v>48.3</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="16">
         <f t="shared" si="0"/>
         <v>2693546.0999999996</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
@@ -4896,13 +4889,13 @@
       <c r="C9" s="6">
         <v>87.4</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="16">
         <f t="shared" si="0"/>
         <v>3405191.4000000004</v>
       </c>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
@@ -4914,13 +4907,13 @@
       <c r="C10" s="6">
         <v>75.7</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="16">
         <f t="shared" si="0"/>
         <v>1708397.6</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
@@ -4932,13 +4925,13 @@
       <c r="C11" s="6">
         <v>77.099999999999994</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="16">
         <f t="shared" si="0"/>
         <v>1671219.5999999999</v>
       </c>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -4950,13 +4943,13 @@
       <c r="C12" s="6">
         <v>95.9</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="16">
         <f t="shared" si="0"/>
         <v>2043724.9000000001</v>
       </c>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
@@ -4968,7 +4961,7 @@
       <c r="C13" s="6">
         <v>96.7</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="16">
         <f t="shared" si="0"/>
         <v>1809257</v>
       </c>
@@ -4983,15 +4976,15 @@
       <c r="C14" s="6">
         <v>66.900000000000006</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="16">
         <f t="shared" si="0"/>
         <v>1175165.4000000001</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="F14" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
@@ -5003,13 +4996,13 @@
       <c r="C15" s="6">
         <v>40.5</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="16">
         <f t="shared" si="0"/>
         <v>415084.5</v>
       </c>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
@@ -5021,13 +5014,13 @@
       <c r="C16" s="6">
         <v>55.9</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="16">
         <f t="shared" si="0"/>
         <v>496615.6</v>
       </c>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
@@ -5039,13 +5032,13 @@
       <c r="C17" s="6">
         <v>96</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="16">
         <f t="shared" si="0"/>
         <v>699072</v>
       </c>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
@@ -5057,13 +5050,13 @@
       <c r="C18" s="6">
         <v>97.1</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="16">
         <f t="shared" si="0"/>
         <v>655813.39999999991</v>
       </c>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
@@ -5075,13 +5068,13 @@
       <c r="C19" s="6">
         <v>72.5</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="16">
         <f t="shared" si="0"/>
         <v>419920</v>
       </c>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
@@ -5093,13 +5086,13 @@
       <c r="C20" s="6">
         <v>102.6</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="16">
         <f t="shared" si="0"/>
         <v>578253.6</v>
       </c>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
@@ -5111,13 +5104,13 @@
       <c r="C21" s="6">
         <v>84.1</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="16">
         <f t="shared" si="0"/>
         <v>443543.39999999997</v>
       </c>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
@@ -5129,13 +5122,13 @@
       <c r="C22" s="6">
         <v>56.9</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="16">
         <f t="shared" si="0"/>
         <v>289621</v>
       </c>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
@@ -5147,13 +5140,13 @@
       <c r="C23" s="6">
         <v>73</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="16">
         <f t="shared" si="0"/>
         <v>346750</v>
       </c>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
@@ -5165,13 +5158,13 @@
       <c r="C24" s="6">
         <v>39.200000000000003</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="16">
         <f t="shared" si="0"/>
         <v>118188.00000000001</v>
       </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
@@ -5183,7 +5176,7 @@
       <c r="C25" s="6">
         <v>124.7</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="16">
         <f t="shared" si="0"/>
         <v>325092.90000000002</v>
       </c>
@@ -5198,7 +5191,7 @@
       <c r="C26" s="6">
         <v>89.1</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="16">
         <f t="shared" si="0"/>
         <v>195129</v>
       </c>
@@ -5213,7 +5206,7 @@
       <c r="C27" s="6">
         <v>97.5</v>
       </c>
-      <c r="D27" s="20">
+      <c r="D27" s="16">
         <f t="shared" si="0"/>
         <v>194805</v>
       </c>
@@ -5228,7 +5221,7 @@
       <c r="C28" s="6">
         <v>72</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="16">
         <f t="shared" si="0"/>
         <v>102960</v>
       </c>
@@ -5243,7 +5236,7 @@
       <c r="C29" s="6">
         <v>56.5</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="16">
         <f t="shared" si="0"/>
         <v>72715.5</v>
       </c>
@@ -5258,7 +5251,7 @@
       <c r="C30" s="6">
         <v>79.2</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="16">
         <f t="shared" si="0"/>
         <v>71359.199999999997</v>
       </c>
@@ -5273,7 +5266,7 @@
       <c r="C31" s="6">
         <v>79.2</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="16">
         <f t="shared" si="0"/>
         <v>65340</v>
       </c>
@@ -5288,7 +5281,7 @@
       <c r="C32" s="6">
         <v>80.099999999999994</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="16">
         <f t="shared" si="0"/>
         <v>56069.999999999993</v>
       </c>
@@ -5303,21 +5296,21 @@
       <c r="C33" s="6">
         <v>90.8</v>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="16">
         <f t="shared" si="0"/>
         <v>41768</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="19">
+      <c r="B34" s="15">
         <f>SUM(B2:B33)</f>
         <v>1271960</v>
       </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="19">
+      <c r="C34" s="7"/>
+      <c r="D34" s="15">
         <f>SUM(D2:D33)</f>
         <v>105491924.3</v>
       </c>
@@ -5338,7 +5331,6 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="18"/>
     <col min="6" max="6" width="14.1640625" customWidth="1"/>
     <col min="7" max="7" width="10.6640625" customWidth="1"/>
     <col min="8" max="8" width="44.5" customWidth="1"/>
@@ -5354,7 +5346,7 @@
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5368,14 +5360,14 @@
       <c r="C2" s="6">
         <v>86.6</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="16">
         <f>B2*C2</f>
         <v>34006434.399999999</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="G2" s="9"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
@@ -5387,14 +5379,14 @@
       <c r="C3" s="6">
         <v>76.099999999999994</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="16">
         <f t="shared" ref="D3:D33" si="0">B3*C3</f>
         <v>15039338.6</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="21">
+      <c r="G3" s="17">
         <f>MAX(C2:C33)-MIN(C2:C33)</f>
         <v>85.5</v>
       </c>
@@ -5413,14 +5405,14 @@
       <c r="C4" s="6">
         <v>90.1</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="16">
         <f t="shared" si="0"/>
         <v>12886372.299999999</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="18">
         <f>QUARTILE(C2:C33,3)-QUARTILE(C2:C33,1)</f>
         <v>19.150000000000006</v>
       </c>
@@ -5439,14 +5431,14 @@
       <c r="C5" s="6">
         <v>84.8</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="16">
         <f t="shared" si="0"/>
         <v>10673521.6</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="18">
         <f>_xlfn.VAR.S(C2:C33)</f>
         <v>350.52221774194021</v>
       </c>
@@ -5465,14 +5457,14 @@
       <c r="C6" s="6">
         <v>88</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="16">
         <f t="shared" si="0"/>
         <v>6596304</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="18">
         <f>STDEV(C2:C33)</f>
         <v>18.722238587891677</v>
       </c>
@@ -5491,14 +5483,14 @@
       <c r="C7" s="6">
         <v>93.7</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="16">
         <f t="shared" si="0"/>
         <v>6195350.2999999998</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="19">
         <f>STDEV(C2:C33)/AVERAGE(C2:C33)</f>
         <v>0.23455940600287128</v>
       </c>
@@ -5517,7 +5509,7 @@
       <c r="C8" s="6">
         <v>48.3</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="16">
         <f t="shared" si="0"/>
         <v>2693546.0999999996</v>
       </c>
@@ -5532,7 +5524,7 @@
       <c r="C9" s="6">
         <v>87.4</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="16">
         <f t="shared" si="0"/>
         <v>3405191.4000000004</v>
       </c>
@@ -5547,15 +5539,15 @@
       <c r="C10" s="6">
         <v>75.7</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="16">
         <f t="shared" si="0"/>
         <v>1708397.6</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="F10" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
     </row>
     <row r="11" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
@@ -5567,13 +5559,13 @@
       <c r="C11" s="6">
         <v>77.099999999999994</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="16">
         <f t="shared" si="0"/>
         <v>1671219.5999999999</v>
       </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
     </row>
     <row r="12" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -5585,13 +5577,13 @@
       <c r="C12" s="6">
         <v>95.9</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="16">
         <f t="shared" si="0"/>
         <v>2043724.9000000001</v>
       </c>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
@@ -5603,13 +5595,13 @@
       <c r="C13" s="6">
         <v>96.7</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="16">
         <f t="shared" si="0"/>
         <v>1809257</v>
       </c>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
     </row>
     <row r="14" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
@@ -5621,13 +5613,13 @@
       <c r="C14" s="6">
         <v>66.900000000000006</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="16">
         <f t="shared" si="0"/>
         <v>1175165.4000000001</v>
       </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
@@ -5639,13 +5631,13 @@
       <c r="C15" s="6">
         <v>40.5</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="16">
         <f t="shared" si="0"/>
         <v>415084.5</v>
       </c>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
@@ -5657,13 +5649,13 @@
       <c r="C16" s="6">
         <v>55.9</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="16">
         <f t="shared" si="0"/>
         <v>496615.6</v>
       </c>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
@@ -5675,13 +5667,13 @@
       <c r="C17" s="6">
         <v>96</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="16">
         <f t="shared" si="0"/>
         <v>699072</v>
       </c>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
@@ -5693,7 +5685,7 @@
       <c r="C18" s="6">
         <v>97.1</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="16">
         <f t="shared" si="0"/>
         <v>655813.39999999991</v>
       </c>
@@ -5708,7 +5700,7 @@
       <c r="C19" s="6">
         <v>72.5</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="16">
         <f t="shared" si="0"/>
         <v>419920</v>
       </c>
@@ -5723,7 +5715,7 @@
       <c r="C20" s="6">
         <v>102.6</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="16">
         <f t="shared" si="0"/>
         <v>578253.6</v>
       </c>
@@ -5738,7 +5730,7 @@
       <c r="C21" s="6">
         <v>84.1</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="16">
         <f t="shared" si="0"/>
         <v>443543.39999999997</v>
       </c>
@@ -5753,7 +5745,7 @@
       <c r="C22" s="6">
         <v>56.9</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="16">
         <f t="shared" si="0"/>
         <v>289621</v>
       </c>
@@ -5768,7 +5760,7 @@
       <c r="C23" s="6">
         <v>73</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="16">
         <f t="shared" si="0"/>
         <v>346750</v>
       </c>
@@ -5783,7 +5775,7 @@
       <c r="C24" s="6">
         <v>39.200000000000003</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="16">
         <f t="shared" si="0"/>
         <v>118188.00000000001</v>
       </c>
@@ -5798,7 +5790,7 @@
       <c r="C25" s="6">
         <v>124.7</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="16">
         <f t="shared" si="0"/>
         <v>325092.90000000002</v>
       </c>
@@ -5813,7 +5805,7 @@
       <c r="C26" s="6">
         <v>89.1</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="16">
         <f t="shared" si="0"/>
         <v>195129</v>
       </c>
@@ -5828,7 +5820,7 @@
       <c r="C27" s="6">
         <v>97.5</v>
       </c>
-      <c r="D27" s="20">
+      <c r="D27" s="16">
         <f t="shared" si="0"/>
         <v>194805</v>
       </c>
@@ -5843,7 +5835,7 @@
       <c r="C28" s="6">
         <v>72</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="16">
         <f t="shared" si="0"/>
         <v>102960</v>
       </c>
@@ -5858,7 +5850,7 @@
       <c r="C29" s="6">
         <v>56.5</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="16">
         <f t="shared" si="0"/>
         <v>72715.5</v>
       </c>
@@ -5873,7 +5865,7 @@
       <c r="C30" s="6">
         <v>79.2</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="16">
         <f t="shared" si="0"/>
         <v>71359.199999999997</v>
       </c>
@@ -5888,7 +5880,7 @@
       <c r="C31" s="6">
         <v>79.2</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="16">
         <f t="shared" si="0"/>
         <v>65340</v>
       </c>
@@ -5903,7 +5895,7 @@
       <c r="C32" s="6">
         <v>80.099999999999994</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="16">
         <f t="shared" si="0"/>
         <v>56069.999999999993</v>
       </c>
@@ -5918,21 +5910,21 @@
       <c r="C33" s="6">
         <v>90.8</v>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="16">
         <f t="shared" si="0"/>
         <v>41768</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="19">
+      <c r="B34" s="15">
         <f>SUM(B2:B33)</f>
         <v>1271960</v>
       </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="19">
+      <c r="C34" s="7"/>
+      <c r="D34" s="15">
         <f>SUM(D2:D33)</f>
         <v>105491924.3</v>
       </c>

</xml_diff>